<commit_message>
Scripts for data comparison
</commit_message>
<xml_diff>
--- a/RQ1 - Non-Refactoring Metrics.xlsx
+++ b/RQ1 - Non-Refactoring Metrics.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Desktop\Software Testing, Quality Assurance &amp; Maintainence\Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Documents\GitHub\SSW567-Fall2023-Group4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE131C8D-FABE-4C26-B2FF-BD6E1E6D28DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38AB4366-46C8-42D2-9B57-513151212F4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="8" xr2:uid="{436870BE-22E1-479F-88F9-25A9F166C2DD}"/>
   </bookViews>
@@ -465,7 +465,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="2">
-        <v>3.9714574438864299</v>
+        <v>7.57</v>
       </c>
       <c r="C2" s="2">
         <v>45</v>
@@ -478,7 +478,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -488,7 +488,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -498,7 +498,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -527,7 +527,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="2">
-        <v>10.512148474192299</v>
+        <v>145.11000000000001</v>
       </c>
       <c r="C2" s="2">
         <v>649</v>
@@ -540,7 +540,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <v>6</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -550,7 +550,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>1</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -560,7 +560,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>12</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -572,6 +572,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1C66934-8D6B-4DEC-B4BF-5AEA454AEE75}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="11.5546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -589,7 +592,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="2">
-        <v>2.8773182137249802</v>
+        <v>106.252981260647</v>
       </c>
       <c r="C2" s="2">
         <v>6575</v>
@@ -602,7 +605,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -622,7 +625,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>1</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -634,6 +637,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D36AD218-FB6D-44F6-8253-C9085E782303}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="11.5546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -651,7 +657,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2">
-        <v>2.9929330299464501</v>
+        <v>34.021294718909701</v>
       </c>
       <c r="C2" s="2">
         <v>225</v>
@@ -664,7 +670,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <v>2</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -674,7 +680,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -684,7 +690,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>3</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -696,6 +702,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1AC0928-AF1F-4231-9732-6AB9984B3E18}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="11.5546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -713,10 +722,10 @@
         <v>0</v>
       </c>
       <c r="B2" s="2">
-        <v>12.638892750929999</v>
+        <v>25.3339011925043</v>
       </c>
       <c r="C2" s="2">
-        <v>99737</v>
+        <v>7418</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -726,7 +735,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -736,7 +745,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -746,7 +755,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -758,6 +767,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ABF248C-CA84-4BAD-9BF8-47A7130AEFB1}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="3" width="11.5546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -772,13 +784,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
-        <v>0</v>
+        <v>1.61111111111111E-2</v>
       </c>
       <c r="B2" s="2">
-        <v>605.89653896686696</v>
+        <v>3624.3976249290199</v>
       </c>
       <c r="C2" s="2">
-        <v>75096.675833333298</v>
+        <v>65639.475555555604</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -788,7 +800,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <v>26.265277777777801</v>
+        <v>1209.7249999999999</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -798,7 +810,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>3.6111111111111101E-3</v>
+        <v>340.84305555555602</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -808,7 +820,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>151.82833333333301</v>
+        <v>3704.6861111111102</v>
       </c>
     </row>
   </sheetData>
@@ -820,6 +832,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F52EE7A-3707-4AE9-A3FE-0EC30B22EE28}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -837,7 +852,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="2">
-        <v>5936.2745165195502</v>
+        <v>262422.27597955702</v>
       </c>
       <c r="C2" s="2">
         <v>5573431</v>
@@ -850,7 +865,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <v>548</v>
+        <v>38164</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -860,7 +875,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>37</v>
+        <v>8270</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -870,7 +885,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>1319</v>
+        <v>216417</v>
       </c>
     </row>
   </sheetData>
@@ -882,6 +897,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED4DDDB4-9498-4CCD-B276-44784DA1A6FB}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="11.5546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -896,13 +914,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="B2" s="2">
-        <v>227.08128371985799</v>
+        <v>262.00766609880702</v>
       </c>
       <c r="C2" s="2">
-        <v>39510</v>
+        <v>2433</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -912,7 +930,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <v>157</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -922,7 +940,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>58</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -932,7 +950,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>272</v>
+        <v>323</v>
       </c>
     </row>
   </sheetData>
@@ -944,6 +962,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F3261F6-AA08-417E-97BF-100DA73C72B6}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="11.5546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -961,10 +982,10 @@
         <v>-1</v>
       </c>
       <c r="B2" s="2">
-        <v>1093.9832210327099</v>
+        <v>4294.1303236797303</v>
       </c>
       <c r="C2" s="2">
-        <v>13408826</v>
+        <v>979462</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -974,7 +995,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <v>12</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -984,7 +1005,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -994,7 +1015,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>52</v>
+        <v>327</v>
       </c>
     </row>
   </sheetData>

</xml_diff>